<commit_message>
IN PROGRESS: updated featurization to include named features that get filtered out by a first pass (looking at features that mostly remain constant and any that have correlation)
</commit_message>
<xml_diff>
--- a/MTGPR_test.xlsx
+++ b/MTGPR_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54AA6691-B367-475D-9FDD-7D255EA894EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91198367-0E44-4427-B7FF-D94A42BE2CC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{535DD4A0-2912-47A9-820B-218FC7178EC0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{535DD4A0-2912-47A9-820B-218FC7178EC0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>T_m</t>
   </si>
@@ -99,19 +99,37 @@
   </si>
   <si>
     <t>C1=CC=C(C=C1)C(=S)N</t>
+  </si>
+  <si>
+    <t>tetrabutylammonium chloride</t>
+  </si>
+  <si>
+    <t>CCCC[N+](CCCC)(CCCC)CCCC.[Cl-]</t>
+  </si>
+  <si>
+    <t>—</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -136,13 +154,38 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -472,14 +515,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB4AABDE-AFF5-4072-A990-39ABD46EABEB}">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
         <v>3</v>
       </c>
@@ -493,7 +536,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -510,7 +553,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -527,11 +570,11 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>13</v>
       </c>
       <c r="D4">
@@ -544,7 +587,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -561,7 +604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -578,11 +621,11 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" t="s">
         <v>17</v>
       </c>
       <c r="D7">
@@ -595,11 +638,11 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" t="s">
         <v>18</v>
       </c>
       <c r="D8">
@@ -612,11 +655,11 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" t="s">
         <v>19</v>
       </c>
       <c r="D9">
@@ -629,7 +672,50 @@
         <v>1</v>
       </c>
     </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10">
+        <v>314.14999999999998</v>
+      </c>
+      <c r="E10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>20.501600000000003</v>
+      </c>
+      <c r="H10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
+      <c r="J10" s="2">
+        <v>-549.4</v>
+      </c>
+      <c r="K10" s="2">
+        <v>21.778888860545631</v>
+      </c>
+      <c r="L10">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="A10">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>AND(F10&gt;0,I10&gt;0,L10&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>OR(F10=0,I10=0,L10=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
switched to using MTGPR via gpytorch and added morgan fingerprints back into the featurization.
</commit_message>
<xml_diff>
--- a/MTGPR_test.xlsx
+++ b/MTGPR_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91198367-0E44-4427-B7FF-D94A42BE2CC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FB2B75A-1069-41BE-9060-7BA2E25DBEE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{535DD4A0-2912-47A9-820B-218FC7178EC0}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{535DD4A0-2912-47A9-820B-218FC7178EC0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,6 +38,91 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Alexander Glotov</author>
+  </authors>
+  <commentList>
+    <comment ref="O2" authorId="0" shapeId="0" xr:uid="{38B88A52-4C56-433F-80C1-0082841D0E2B}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://matweb.com/search/datasheet.aspx?MatGUID=3118b2052ace4835a6d73687613def66&amp;ckck=1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N4" authorId="0" shapeId="0" xr:uid="{FBF27A95-B6A7-44EB-9970-EEADCAF92B12}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+1)https://iris.unito.it/bitstream/2318/1995351/2/Dematteis%20-%20PhD%20Thesis%20-%20DEF_REFEREE.pdf</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O6" authorId="0" shapeId="0" xr:uid="{C2EC2B03-0223-48AF-894B-A38079C87F08}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://www.sciencedirect.com/science/article/abs/pii/S0040603115003354
+2)https://www.sciencedirect.com/science/article/pii/S0016236125036129</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
@@ -117,7 +202,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -130,6 +215,32 @@
       <color rgb="FF000000"/>
       <name val="Aptos"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -514,15 +625,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB4AABDE-AFF5-4072-A990-39ABD46EABEB}">
-  <dimension ref="A1:L10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB4AABDE-AFF5-4072-A990-39ABD46EABEB}">
+  <dimension ref="A1:O10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
         <v>3</v>
       </c>
@@ -536,7 +647,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -544,16 +655,25 @@
         <v>5</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>559.15</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <f>N2/1000</f>
+        <v>7.14</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <f>O2/1000</f>
+        <v>-190.8</v>
+      </c>
+      <c r="N2">
+        <f>AVERAGE(7.56,6.72)*1000</f>
+        <v>7140</v>
+      </c>
+      <c r="O2">
+        <v>-190800</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -561,16 +681,25 @@
         <v>7</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>673.15</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <f t="shared" ref="G3:G9" si="0">N3/1000</f>
+        <v>16</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <f t="shared" ref="J3:J9" si="1">O3/1000</f>
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <f>AVERAGE(16.9,15.1)*1000</f>
+        <v>16000</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -578,16 +707,25 @@
         <v>13</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>878.15</v>
       </c>
       <c r="G4">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>19.2</v>
       </c>
       <c r="J4">
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <f>AVERAGE(19.2)*1000</f>
+        <v>19200</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -595,16 +733,24 @@
         <v>9</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>397.15</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>15.8</v>
       </c>
       <c r="J5">
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>-395</v>
+      </c>
+      <c r="N5">
+        <v>15800</v>
+      </c>
+      <c r="O5">
+        <v>-395000</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -612,16 +758,24 @@
         <v>11</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>381.15</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>14.6</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>-133.4</v>
+      </c>
+      <c r="N6">
+        <v>14600</v>
+      </c>
+      <c r="O6">
+        <v>-133400</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -629,16 +783,24 @@
         <v>17</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>449.7</v>
       </c>
       <c r="G7">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>13.597</v>
       </c>
       <c r="J7">
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>-89.1</v>
+      </c>
+      <c r="N7">
+        <v>13597</v>
+      </c>
+      <c r="O7">
+        <v>-89100</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -646,16 +808,24 @@
         <v>18</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>385.7</v>
       </c>
       <c r="G8">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>18.36</v>
       </c>
       <c r="J8">
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>-73.010000000000005</v>
+      </c>
+      <c r="N8">
+        <v>18360</v>
+      </c>
+      <c r="O8">
+        <v>-73010</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -663,16 +833,24 @@
         <v>19</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>387.15</v>
       </c>
       <c r="G9">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>17.73</v>
       </c>
       <c r="J9">
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="N9">
+        <v>17730</v>
+      </c>
+      <c r="O9">
+        <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>20</v>
       </c>
@@ -717,5 +895,6 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>